<commit_message>
Finalize webhook replay Windows reproduction
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="Ra942108734b44f5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="Rc9d0ccba43e04bed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -429,35 +429,19 @@
         <x:v>intake_decisions.csv保持输入顺序；replay_queue.jsonl按scheduled_at_utc和event_id升序；endpoint_handoff.csv保持策略顺序</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="33" customHeight="1">
+    <x:row r="16" ht="48" customHeight="1">
       <x:c r="A16" s="5" t="str">
-        <x:v>失败保全</x:v>
+        <x:v>完成条件</x:v>
       </x:c>
       <x:c r="B16" s="5" t="str">
-        <x:v>业务输入或合同无法读取时返回非0，首次失败不留下半成品，已有完整交付不被部分结果替换</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="48" customHeight="1">
+        <x:v>npm run rebuild返回0，四个目标路径存在，13条事件均有唯一终态，排队事件在裁决台账与重放队列之间一一对应</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="33" customHeight="1">
       <x:c r="A17" s="5" t="str">
-        <x:v>完成条件</x:v>
+        <x:v>不适合作为评分点的内容</x:v>
       </x:c>
       <x:c r="B17" s="5" t="str">
-        <x:v>npm run rebuild返回0，四个目标路径存在，13条事件均有唯一终态，排队事件在裁决台账与重放队列之间一一对应</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="48" customHeight="1">
-      <x:c r="A18" s="5" t="str">
-        <x:v>可验证点</x:v>
-      </x:c>
-      <x:c r="B18" s="5" t="str">
-        <x:v>crypto.verify运行语义；13条裁决映射；4条队列记录与退避时刻；三个端点的计数和最早时刻；失败时的原子发布行为</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="33" customHeight="1">
-      <x:c r="A19" s="5" t="str">
-        <x:v>不适合作为评分点的内容</x:v>
-      </x:c>
-      <x:c r="B19" s="5" t="str">
         <x:v>函数拆分、变量名、注释风格、JSON键序、CSV必要引号、LF或CRLF行尾以及临时目录名称</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Generalize specification completion rule
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="Rc9d0ccba43e04bed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="Rd9e796d0a3614f6d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -434,7 +434,7 @@
         <x:v>完成条件</x:v>
       </x:c>
       <x:c r="B16" s="5" t="str">
-        <x:v>npm run rebuild返回0，四个目标路径存在，13条事件均有唯一终态，排队事件在裁决台账与重放队列之间一一对应</x:v>
+        <x:v>npm run rebuild返回0，四个目标路径存在，每条非空输入事件均有唯一终态，排队事件在裁决台账与重放队列之间一一对应</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="33" customHeight="1">

</xml_diff>